<commit_message>
large commit of stuff
</commit_message>
<xml_diff>
--- a/data/Daten_DA.xlsx
+++ b/data/Daten_DA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/felixwegener/freelancing/data-analytics-project/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32E54865-604D-B245-A508-31661C02C27D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3F43CE1-1937-2B42-9423-EE193815ED23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="36000" windowHeight="21100" xr2:uid="{9E9AB009-95EC-6B4D-94A0-22510EA99775}"/>
   </bookViews>
@@ -224,7 +224,7 @@
     <t>urb_ceduc_page_linear_2_0</t>
   </si>
   <si>
-    <t>total nr of people per city</t>
+    <t>total nr of people per city, with summed rows per country</t>
   </si>
 </sst>
 </file>

</xml_diff>